<commit_message>
Update IGs +Add  YAML Version
</commit_message>
<xml_diff>
--- a/tools/excel/anssi/anssi-mon-aide-cyber.xlsx
+++ b/tools/excel/anssi/anssi-mon-aide-cyber.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\tarkadia\projects\intuitem\ciso-assistant-community\tools\excel\anssi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42DB6B3C-31CB-44A6-BCD4-EAB5DE2615C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC852140-3FF0-4DF8-BAF9-457CE2E6F1CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1485" yWindow="-15870" windowWidth="25440" windowHeight="15990" tabRatio="882" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="26400" yWindow="-4008" windowWidth="25404" windowHeight="12228" tabRatio="882" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="621">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="612">
   <si>
     <t>type</t>
   </si>
@@ -203,16 +203,10 @@
     <t>contexte-cyber-attaque-subie-oui-tiroir-type</t>
   </si>
   <si>
-    <t>_Q8.1_DEPENDS_ON_contexte-cyber-attaque-subie</t>
-  </si>
-  <si>
     <t>Si oui, de quel type ?</t>
   </si>
   <si>
     <t>contexte-cyber-attaque-subie-tiroir-plainte</t>
-  </si>
-  <si>
-    <t>_Q8.2_DEPENDS_ON_contexte-cyber-attaque-subie</t>
   </si>
   <si>
     <t>Si Oui : avez-vous déposé plainte ou réalisé un signalement auprès d'un service judiciaire ?</t>
@@ -518,9 +512,6 @@
     <t>securite-infrastructure-pare-feu-deploye-oui-tiroir-interconnexions-protegees</t>
   </si>
   <si>
-    <t>_Q33.1_DEPENDS_ON_securite-infrastructure-pare-feu-deploye</t>
-  </si>
-  <si>
     <t>Est-ce que seuls les flux entrants et sortants strictement nécessaires entre Internet et le système d'information (ou autres réseaux externes) sont autorisés ?</t>
   </si>
   <si>
@@ -529,9 +520,6 @@
   </si>
   <si>
     <t>securite-infrastructure-pare-feu-deploye-oui-tiroir-logs-stockes</t>
-  </si>
-  <si>
-    <t>_Q33.2_DEPENDS_ON_securite-infrastructure-pare-feu-deploye</t>
   </si>
   <si>
     <t>Les journaux des flux entrants, sortants et bloqués (générés par le pare-feu) sont-ils stockés ?</t>
@@ -670,9 +658,6 @@
     <t>reaction-sauvegardes-donnees-realisees-oui-ponctuellement-tiroir-environnement-isole</t>
   </si>
   <si>
-    <t>_Q44.1_DEPENDS_ON_reaction-sauvegardes-donnees-realisees</t>
-  </si>
-  <si>
     <t>Existe-t-il au moins un jeu de sauvegarde des données critiques stockées dans un environnement isolé du réseau bureautique interne ou "hors ligne" ?</t>
   </si>
   <si>
@@ -682,9 +667,6 @@
     <t>reaction-sauvegardes-donnees-realisees-oui-ponctuellement-tiroir-sauvegarde-testee-regulierement</t>
   </si>
   <si>
-    <t>_Q44.2_DEPENDS_ON_reaction-sauvegardes-donnees-realisees</t>
-  </si>
-  <si>
     <t>Si "Oui" : La restauration des sauvegardes de toutes vos données critiques est-elle testée régulièrement ?</t>
   </si>
   <si>
@@ -694,19 +676,10 @@
     <t>reaction-sauvegardes-donnees-realisees-oui-automatique-et-reguliere-tiroir-environnement-isole</t>
   </si>
   <si>
-    <t>_Q44.3_DEPENDS_ON_reaction-sauvegardes-donnees-realisees</t>
-  </si>
-  <si>
-    <t>Existe-t-il au moins un jeu de sauvegarde des données critiques stockées dans un environnement isolé du réseau bureautique interne ou "hors ligne"</t>
-  </si>
-  <si>
     <t>1:reaction-sauvegardes-donnees-realisees-oui-automatique-et-reguliere-tiroir-environnement-isole_niveau1</t>
   </si>
   <si>
     <t>reaction-sauvegardes-donnees-realisees-oui-automatique-et-reguliere-tiroir-sauvegarde-testee-regulierement</t>
-  </si>
-  <si>
-    <t>_Q44.4_DEPENDS_ON_reaction-sauvegardes-donnees-realisees</t>
   </si>
   <si>
     <t>La restauration des sauvegardes de toutes vos données critiques est-elle testée régulièrement ?</t>
@@ -910,11 +883,6 @@
 _DEPENDS_ON_contexte-opere-systemes-information-industriels</t>
   </si>
   <si>
-    <t>/
-/
-_Q8.1_DEPENDS_ON_contexte-cyber-attaque-subie, _Q8.2_DEPENDS_ON_contexte-cyber-attaque-subie</t>
-  </si>
-  <si>
     <t>multiple_choice</t>
   </si>
   <si>
@@ -1068,11 +1036,6 @@
 Oui, un outil de type EDR a été mis en place et ses alertes sont systématiquement traitées</t>
   </si>
   <si>
-    <t>/
-/
-_Q33.1_DEPENDS_ON_securite-infrastructure-pare-feu-deploye, _Q33.2_DEPENDS_ON_securite-infrastructure-pare-feu-deploye</t>
-  </si>
-  <si>
     <t>Je ne sais pas
 Non
 Oui
@@ -1143,12 +1106,6 @@
 Des sauvegardes des données sont réalisées de manière automatique et régulière</t>
   </si>
   <si>
-    <t>/
-/
-_Q44.1_DEPENDS_ON_reaction-sauvegardes-donnees-realisees, _Q44.2_DEPENDS_ON_reaction-sauvegardes-donnees-realisees
-_Q44.3_DEPENDS_ON_reaction-sauvegardes-donnees-realisees, _Q44.4_DEPENDS_ON_reaction-sauvegardes-donnees-realisees</t>
-  </si>
-  <si>
     <t>Je ne sais pas
 Non
 Oui, nous avons formalisé une fiche réflexe dédiée
@@ -1710,42 +1667,6 @@
 #555555
 #8B0000
 /</t>
-  </si>
-  <si>
-    <t>Question 33.1 dépendante de la Question 33</t>
-  </si>
-  <si>
-    <t>Question 33.2 dépendante de la Question 33</t>
-  </si>
-  <si>
-    <t>Question 44.1 dépendante de la Question 44</t>
-  </si>
-  <si>
-    <t>Question 44.2 dépendante de la Question 44</t>
-  </si>
-  <si>
-    <t>Question 44.3 dépendante de la Question 44</t>
-  </si>
-  <si>
-    <t>Question 44.4 dépendante de la Question 44</t>
-  </si>
-  <si>
-    <t>Question 8.1 dépendante de la Question 8</t>
-  </si>
-  <si>
-    <t>Question 8.2 dépendante de la Question 8</t>
-  </si>
-  <si>
-    <t>Questions dépendantes de la Question 7</t>
-  </si>
-  <si>
-    <t>Questions dépendantes de la Question 6</t>
-  </si>
-  <si>
-    <t>Questions dépendantes de la Question 5</t>
-  </si>
-  <si>
-    <t>Questions dépendantes de la Question</t>
   </si>
   <si>
     <t>MonAideCyber aide les entités publiques et privées sensibilisées à la sécurité informatique à passer à l’action. Le dispositif MonAideCyber est développé par l'Agence Nationale de la Sécurité des Systèmes d'Information, en lien avec BetaGouv et la Direction interministérielle du numérique.
@@ -2800,6 +2721,58 @@
   </si>
   <si>
     <t>Question 45</t>
+  </si>
+  <si>
+    <t>Dépendance à attaque subie</t>
+  </si>
+  <si>
+    <t>Dépendance à pare-feu déployé</t>
+  </si>
+  <si>
+    <t>Dépendance à sauvegardes ponctuelles</t>
+  </si>
+  <si>
+    <t>Dépendance à sauvegardes régulières</t>
+  </si>
+  <si>
+    <t>Dépendance à SI industriel</t>
+  </si>
+  <si>
+    <t>Dépendance à activités R&amp;D</t>
+  </si>
+  <si>
+    <t>Dépendance à postes de travail dans entité</t>
+  </si>
+  <si>
+    <t>Dépendance à postes de travail dans organisation</t>
+  </si>
+  <si>
+    <t>_DEPENDS_ON_contexte-cyber-attaque-subie</t>
+  </si>
+  <si>
+    <t>_DEPENDS_ON_securite-infrastructure-pare-feu-deploye</t>
+  </si>
+  <si>
+    <t>_DEPENDS_ON_reaction-sauvegardes-donnees-realisees-ponctuellement</t>
+  </si>
+  <si>
+    <t>_DEPENDS_ON_reaction-sauvegardes-donnees-realisees-regulierement</t>
+  </si>
+  <si>
+    <t>/
+/
+_DEPENDS_ON_reaction-sauvegardes-donnees-realisees-ponctuellement
+_DEPENDS_ON_reaction-sauvegardes-donnees-realisees-regulierement</t>
+  </si>
+  <si>
+    <t>/
+/
+_DEPENDS_ON_securite-infrastructure-pare-feu-deploye</t>
+  </si>
+  <si>
+    <t>/
+/
+_DEPENDS_ON_contexte-cyber-attaque-subie</t>
   </si>
 </sst>
 </file>
@@ -2835,7 +2808,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -2844,7 +2817,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3207,7 +3179,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>458</v>
+        <v>434</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="158.4" x14ac:dyDescent="0.3">
@@ -3215,7 +3187,7 @@
         <v>13</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>565</v>
+        <v>541</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -3252,7 +3224,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>430</v>
+        <v>418</v>
       </c>
     </row>
   </sheetData>
@@ -3270,10 +3242,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>431</v>
+        <v>419</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>432</v>
+        <v>420</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -3281,7 +3253,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -3343,7 +3315,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>458</v>
+        <v>434</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -3379,7 +3351,7 @@
     <col min="5" max="5" width="88.44140625" style="3" customWidth="1"/>
     <col min="6" max="6" width="129.21875" style="3" customWidth="1"/>
     <col min="7" max="7" width="14.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="63.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="86.77734375" style="3" customWidth="1"/>
     <col min="9" max="9" width="152.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="95.44140625" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="117.109375" style="3" bestFit="1" customWidth="1"/>
@@ -3394,7 +3366,7 @@
         <v>27</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>459</v>
+        <v>435</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>10</v>
@@ -3420,8 +3392,8 @@
       <c r="K1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="4" t="s">
-        <v>567</v>
+      <c r="L1" s="1" t="s">
+        <v>543</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -3444,7 +3416,7 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="4"/>
+      <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -3459,7 +3431,7 @@
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>460</v>
+        <v>436</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2" t="s">
@@ -3472,8 +3444,8 @@
         <v>39</v>
       </c>
       <c r="K3" s="2"/>
-      <c r="L3" s="4" t="s">
-        <v>568</v>
+      <c r="L3" s="1" t="s">
+        <v>544</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -3489,7 +3461,7 @@
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>461</v>
+        <v>437</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2" t="s">
@@ -3502,8 +3474,8 @@
         <v>42</v>
       </c>
       <c r="K4" s="2"/>
-      <c r="L4" s="4" t="s">
-        <v>569</v>
+      <c r="L4" s="1" t="s">
+        <v>545</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -3530,8 +3502,8 @@
         <v>44</v>
       </c>
       <c r="K5" s="2"/>
-      <c r="L5" s="4" t="s">
-        <v>570</v>
+      <c r="L5" s="1" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -3558,8 +3530,8 @@
         <v>46</v>
       </c>
       <c r="K6" s="2"/>
-      <c r="L6" s="4" t="s">
-        <v>571</v>
+      <c r="L6" s="1" t="s">
+        <v>547</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -3575,7 +3547,7 @@
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
-        <v>462</v>
+        <v>438</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2" t="s">
@@ -3588,8 +3560,8 @@
         <v>48</v>
       </c>
       <c r="K7" s="2"/>
-      <c r="L7" s="4" t="s">
-        <v>572</v>
+      <c r="L7" s="1" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
@@ -3605,7 +3577,7 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>463</v>
+        <v>439</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2" t="s">
@@ -3618,8 +3590,8 @@
         <v>50</v>
       </c>
       <c r="K8" s="2"/>
-      <c r="L8" s="4" t="s">
-        <v>573</v>
+      <c r="L8" s="1" t="s">
+        <v>549</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="115.2" x14ac:dyDescent="0.3">
@@ -3635,7 +3607,7 @@
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
-        <v>464</v>
+        <v>440</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2" t="s">
@@ -3648,8 +3620,8 @@
         <v>52</v>
       </c>
       <c r="K9" s="2"/>
-      <c r="L9" s="4" t="s">
-        <v>574</v>
+      <c r="L9" s="1" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -3665,7 +3637,7 @@
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
-        <v>465</v>
+        <v>441</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2" t="s">
@@ -3678,8 +3650,8 @@
         <v>54</v>
       </c>
       <c r="K10" s="2"/>
-      <c r="L10" s="4" t="s">
-        <v>575</v>
+      <c r="L10" s="1" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -3687,7 +3659,7 @@
         <v>37</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>566</v>
+        <v>542</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>56</v>
@@ -3697,17 +3669,17 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>56</v>
       </c>
       <c r="K11" s="2"/>
-      <c r="L11" s="4" t="s">
-        <v>576</v>
+      <c r="L11" s="1" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
@@ -3715,27 +3687,27 @@
         <v>37</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>566</v>
+        <v>542</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2" t="s">
-        <v>60</v>
+        <v>605</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K12" s="2"/>
-      <c r="L12" s="4" t="s">
-        <v>577</v>
+      <c r="L12" s="1" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -3744,13 +3716,13 @@
         <v>5</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -3758,7 +3730,7 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
-      <c r="L13" s="4"/>
+      <c r="L13" s="1"/>
     </row>
     <row r="14" spans="1:12" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
@@ -3768,28 +3740,28 @@
         <v>38</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>466</v>
+        <v>442</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J14" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K14" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="K14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="L14" s="4" t="s">
-        <v>578</v>
+      <c r="L14" s="1" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="115.2" x14ac:dyDescent="0.3">
@@ -3800,28 +3772,28 @@
         <v>38</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
-        <v>467</v>
+        <v>443</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J15" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="K15" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="L15" s="4" t="s">
-        <v>579</v>
+      <c r="L15" s="1" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
@@ -3832,28 +3804,28 @@
         <v>38</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
-        <v>468</v>
+        <v>444</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="K16" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="I16" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="L16" s="4" t="s">
-        <v>580</v>
+      <c r="L16" s="1" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="172.8" x14ac:dyDescent="0.3">
@@ -3864,28 +3836,28 @@
         <v>38</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2" t="s">
-        <v>469</v>
+        <v>445</v>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J17" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="K17" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="L17" s="4" t="s">
-        <v>581</v>
+      <c r="L17" s="1" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -3896,28 +3868,28 @@
         <v>38</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>470</v>
+        <v>446</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="J18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K18" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="L18" s="4" t="s">
-        <v>582</v>
+      <c r="L18" s="1" t="s">
+        <v>558</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="158.4" x14ac:dyDescent="0.3">
@@ -3928,28 +3900,28 @@
         <v>38</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2" t="s">
-        <v>471</v>
+        <v>447</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J19" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K19" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="K19" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="L19" s="4" t="s">
-        <v>583</v>
+      <c r="L19" s="1" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -3958,13 +3930,13 @@
         <v>5</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -3972,7 +3944,7 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
-      <c r="L20" s="4"/>
+      <c r="L20" s="1"/>
     </row>
     <row r="21" spans="1:12" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
@@ -3982,28 +3954,28 @@
         <v>38</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2" t="s">
-        <v>472</v>
+        <v>448</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="K21" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="I21" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="L21" s="4" t="s">
-        <v>584</v>
+      <c r="L21" s="1" t="s">
+        <v>560</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
@@ -4014,28 +3986,28 @@
         <v>38</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
-        <v>473</v>
+        <v>449</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="K22" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="I22" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="L22" s="4" t="s">
-        <v>585</v>
+      <c r="L22" s="1" t="s">
+        <v>561</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
@@ -4046,28 +4018,28 @@
         <v>38</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2" t="s">
-        <v>473</v>
+        <v>449</v>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J23" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="K23" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="K23" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="L23" s="4" t="s">
-        <v>586</v>
+      <c r="L23" s="1" t="s">
+        <v>562</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
@@ -4078,28 +4050,28 @@
         <v>38</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2" t="s">
-        <v>474</v>
+        <v>450</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="J24" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K24" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="K24" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="L24" s="4" t="s">
-        <v>587</v>
+      <c r="L24" s="1" t="s">
+        <v>563</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
@@ -4110,28 +4082,28 @@
         <v>38</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
-        <v>475</v>
+        <v>451</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J25" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="K25" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="K25" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="L25" s="4" t="s">
-        <v>588</v>
+      <c r="L25" s="1" t="s">
+        <v>564</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -4142,28 +4114,28 @@
         <v>38</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2" t="s">
-        <v>476</v>
+        <v>452</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J26" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="K26" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="K26" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="L26" s="4" t="s">
-        <v>589</v>
+      <c r="L26" s="1" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="144" x14ac:dyDescent="0.3">
@@ -4174,28 +4146,28 @@
         <v>38</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2" t="s">
-        <v>477</v>
+        <v>453</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J27" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="K27" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="K27" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="L27" s="4" t="s">
-        <v>590</v>
+      <c r="L27" s="1" t="s">
+        <v>566</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="172.8" x14ac:dyDescent="0.3">
@@ -4206,28 +4178,28 @@
         <v>38</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2" t="s">
-        <v>478</v>
+        <v>454</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="J28" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="K28" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="K28" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L28" s="4" t="s">
-        <v>591</v>
+      <c r="L28" s="1" t="s">
+        <v>567</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
@@ -4238,28 +4210,28 @@
         <v>38</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2" t="s">
-        <v>479</v>
+        <v>455</v>
       </c>
       <c r="G29" s="2"/>
       <c r="H29" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J29" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K29" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="K29" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="L29" s="4" t="s">
-        <v>592</v>
+      <c r="L29" s="1" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -4270,28 +4242,28 @@
         <v>38</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2" t="s">
-        <v>480</v>
+        <v>456</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J30" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="K30" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="K30" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="L30" s="4" t="s">
-        <v>593</v>
+      <c r="L30" s="1" t="s">
+        <v>569</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="115.2" x14ac:dyDescent="0.3">
@@ -4302,28 +4274,28 @@
         <v>38</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2" t="s">
-        <v>481</v>
+        <v>457</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="J31" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="K31" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="K31" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="L31" s="4" t="s">
-        <v>594</v>
+      <c r="L31" s="1" t="s">
+        <v>570</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -4332,13 +4304,13 @@
         <v>5</v>
       </c>
       <c r="C32" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
@@ -4346,7 +4318,7 @@
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
-      <c r="L32" s="4"/>
+      <c r="L32" s="1"/>
     </row>
     <row r="33" spans="1:12" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
@@ -4356,28 +4328,28 @@
         <v>38</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
-        <v>482</v>
+        <v>458</v>
       </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J33" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="K33" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="K33" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="L33" s="4" t="s">
-        <v>595</v>
+      <c r="L33" s="1" t="s">
+        <v>571</v>
       </c>
     </row>
     <row r="34" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -4388,28 +4360,28 @@
         <v>38</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2" t="s">
-        <v>480</v>
+        <v>456</v>
       </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J34" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="K34" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="K34" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="L34" s="4" t="s">
-        <v>596</v>
+      <c r="L34" s="1" t="s">
+        <v>572</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
@@ -4420,28 +4392,28 @@
         <v>38</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
       <c r="F35" s="2" t="s">
-        <v>483</v>
+        <v>459</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="J35" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="K35" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="K35" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="L35" s="4" t="s">
-        <v>597</v>
+      <c r="L35" s="1" t="s">
+        <v>573</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -4452,28 +4424,28 @@
         <v>38</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
       <c r="F36" s="2" t="s">
-        <v>480</v>
+        <v>456</v>
       </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J36" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="K36" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="K36" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="L36" s="4" t="s">
-        <v>598</v>
+      <c r="L36" s="1" t="s">
+        <v>574</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
@@ -4484,28 +4456,28 @@
         <v>38</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
       <c r="F37" s="2" t="s">
-        <v>484</v>
+        <v>460</v>
       </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="J37" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="K37" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="K37" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="L37" s="4" t="s">
-        <v>599</v>
+      <c r="L37" s="1" t="s">
+        <v>575</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -4516,28 +4488,28 @@
         <v>38</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
       <c r="F38" s="2" t="s">
-        <v>485</v>
+        <v>461</v>
       </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J38" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="K38" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="K38" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="L38" s="4" t="s">
-        <v>600</v>
+      <c r="L38" s="1" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="39" spans="1:12" ht="216" x14ac:dyDescent="0.3">
@@ -4548,28 +4520,28 @@
         <v>38</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
       <c r="F39" s="2" t="s">
-        <v>486</v>
+        <v>462</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J39" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="K39" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="K39" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="L39" s="4" t="s">
-        <v>601</v>
+      <c r="L39" s="1" t="s">
+        <v>577</v>
       </c>
     </row>
     <row r="40" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -4578,13 +4550,13 @@
         <v>5</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>150</v>
       </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
@@ -4592,7 +4564,7 @@
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
-      <c r="L40" s="4"/>
+      <c r="L40" s="1"/>
     </row>
     <row r="41" spans="1:12" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
@@ -4602,28 +4574,28 @@
         <v>38</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
       <c r="F41" s="2" t="s">
-        <v>487</v>
+        <v>463</v>
       </c>
       <c r="G41" s="2"/>
       <c r="H41" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="J41" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="K41" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="K41" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="L41" s="4" t="s">
-        <v>602</v>
+      <c r="L41" s="1" t="s">
+        <v>578</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -4631,29 +4603,29 @@
         <v>37</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>566</v>
+        <v>542</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
       <c r="H42" s="2" t="s">
-        <v>155</v>
+        <v>606</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="J42" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="K42" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="K42" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="L42" s="4" t="s">
-        <v>603</v>
+      <c r="L42" s="1" t="s">
+        <v>579</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.3">
@@ -4661,29 +4633,29 @@
         <v>37</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>566</v>
+        <v>542</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
       <c r="H43" s="2" t="s">
-        <v>159</v>
+        <v>606</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="L43" s="4" t="s">
-        <v>604</v>
+        <v>157</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>580</v>
       </c>
     </row>
     <row r="44" spans="1:12" ht="115.2" x14ac:dyDescent="0.3">
@@ -4694,28 +4666,28 @@
         <v>38</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
       <c r="F44" s="2" t="s">
-        <v>488</v>
+        <v>464</v>
       </c>
       <c r="G44" s="2"/>
       <c r="H44" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="L44" s="4" t="s">
-        <v>605</v>
+        <v>160</v>
+      </c>
+      <c r="L44" s="1" t="s">
+        <v>581</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
@@ -4726,28 +4698,28 @@
         <v>38</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
       <c r="F45" s="2" t="s">
-        <v>489</v>
+        <v>465</v>
       </c>
       <c r="G45" s="2"/>
       <c r="H45" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="L45" s="4" t="s">
-        <v>606</v>
+        <v>163</v>
+      </c>
+      <c r="L45" s="1" t="s">
+        <v>582</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="187.2" x14ac:dyDescent="0.3">
@@ -4758,28 +4730,28 @@
         <v>38</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
       <c r="F46" s="2" t="s">
-        <v>490</v>
+        <v>466</v>
       </c>
       <c r="G46" s="2"/>
       <c r="H46" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="L46" s="4" t="s">
-        <v>607</v>
+        <v>166</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>583</v>
       </c>
     </row>
     <row r="47" spans="1:12" ht="129.6" x14ac:dyDescent="0.3">
@@ -4790,28 +4762,28 @@
         <v>38</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
       <c r="F47" s="2" t="s">
-        <v>491</v>
+        <v>467</v>
       </c>
       <c r="G47" s="2"/>
       <c r="H47" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="L47" s="4" t="s">
-        <v>608</v>
+        <v>169</v>
+      </c>
+      <c r="L47" s="1" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="115.2" x14ac:dyDescent="0.3">
@@ -4822,28 +4794,28 @@
         <v>38</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2" t="s">
-        <v>492</v>
+        <v>468</v>
       </c>
       <c r="G48" s="2"/>
       <c r="H48" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="L48" s="4" t="s">
-        <v>609</v>
+        <v>172</v>
+      </c>
+      <c r="L48" s="1" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="49" spans="1:12" ht="144" x14ac:dyDescent="0.3">
@@ -4854,28 +4826,28 @@
         <v>38</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="2" t="s">
-        <v>493</v>
+        <v>469</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="L49" s="4" t="s">
-        <v>610</v>
+        <v>175</v>
+      </c>
+      <c r="L49" s="1" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -4884,13 +4856,13 @@
         <v>5</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
@@ -4898,7 +4870,7 @@
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
-      <c r="L50" s="4"/>
+      <c r="L50" s="1"/>
     </row>
     <row r="51" spans="1:12" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
@@ -4908,28 +4880,28 @@
         <v>38</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
       <c r="F51" s="2" t="s">
-        <v>494</v>
+        <v>470</v>
       </c>
       <c r="G51" s="2"/>
       <c r="H51" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="L51" s="4" t="s">
-        <v>611</v>
+        <v>181</v>
+      </c>
+      <c r="L51" s="1" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="52" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
@@ -4940,28 +4912,28 @@
         <v>38</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
       <c r="F52" s="2" t="s">
-        <v>495</v>
+        <v>471</v>
       </c>
       <c r="G52" s="2"/>
       <c r="H52" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="L52" s="4" t="s">
-        <v>612</v>
+        <v>184</v>
+      </c>
+      <c r="L52" s="1" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="53" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -4972,26 +4944,26 @@
         <v>38</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
       <c r="H53" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="L53" s="4" t="s">
-        <v>613</v>
+        <v>187</v>
+      </c>
+      <c r="L53" s="1" t="s">
+        <v>589</v>
       </c>
     </row>
     <row r="54" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -5000,13 +4972,13 @@
         <v>5</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
@@ -5014,7 +4986,7 @@
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
-      <c r="L54" s="4"/>
+      <c r="L54" s="1"/>
     </row>
     <row r="55" spans="1:12" ht="144" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
@@ -5024,28 +4996,28 @@
         <v>38</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
       <c r="F55" s="2" t="s">
-        <v>496</v>
+        <v>472</v>
       </c>
       <c r="G55" s="2"/>
       <c r="H55" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="L55" s="4" t="s">
-        <v>614</v>
+        <v>193</v>
+      </c>
+      <c r="L55" s="1" t="s">
+        <v>590</v>
       </c>
     </row>
     <row r="56" spans="1:12" ht="187.2" x14ac:dyDescent="0.3">
@@ -5056,28 +5028,28 @@
         <v>38</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D56" s="2"/>
       <c r="E56" s="2"/>
       <c r="F56" s="2" t="s">
-        <v>497</v>
+        <v>473</v>
       </c>
       <c r="G56" s="2"/>
       <c r="H56" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="L56" s="4" t="s">
-        <v>615</v>
+        <v>196</v>
+      </c>
+      <c r="L56" s="1" t="s">
+        <v>591</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.3">
@@ -5085,29 +5057,29 @@
         <v>37</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>566</v>
+        <v>542</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
       <c r="H57" s="2" t="s">
-        <v>202</v>
+        <v>607</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="L57" s="4" t="s">
-        <v>616</v>
+        <v>199</v>
+      </c>
+      <c r="L57" s="1" t="s">
+        <v>592</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.3">
@@ -5115,29 +5087,29 @@
         <v>37</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>566</v>
+        <v>542</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
       <c r="H58" s="2" t="s">
-        <v>206</v>
+        <v>607</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="L58" s="4" t="s">
-        <v>617</v>
+        <v>202</v>
+      </c>
+      <c r="L58" s="1" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.3">
@@ -5145,29 +5117,29 @@
         <v>37</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>566</v>
+        <v>542</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
       <c r="G59" s="2"/>
       <c r="H59" s="2" t="s">
-        <v>210</v>
+        <v>608</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>211</v>
+        <v>198</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="L59" s="4" t="s">
-        <v>618</v>
+        <v>204</v>
+      </c>
+      <c r="L59" s="1" t="s">
+        <v>594</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.3">
@@ -5175,29 +5147,29 @@
         <v>37</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>566</v>
+        <v>542</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
       <c r="H60" s="2" t="s">
-        <v>214</v>
+        <v>608</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="L60" s="4" t="s">
-        <v>619</v>
+        <v>207</v>
+      </c>
+      <c r="L60" s="1" t="s">
+        <v>595</v>
       </c>
     </row>
     <row r="61" spans="1:12" ht="72" x14ac:dyDescent="0.3">
@@ -5208,28 +5180,28 @@
         <v>38</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="D61" s="2"/>
       <c r="E61" s="2"/>
       <c r="F61" s="2" t="s">
-        <v>498</v>
+        <v>474</v>
       </c>
       <c r="G61" s="2"/>
       <c r="H61" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="L61" s="4" t="s">
-        <v>620</v>
+        <v>210</v>
+      </c>
+      <c r="L61" s="1" t="s">
+        <v>596</v>
       </c>
     </row>
   </sheetData>
@@ -5247,7 +5219,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -5272,28 +5244,28 @@
     <col min="2" max="2" width="15.88671875" style="3" customWidth="1"/>
     <col min="3" max="3" width="139.33203125" style="3" customWidth="1"/>
     <col min="4" max="4" width="12.44140625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="131.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="200.6640625" style="3" customWidth="1"/>
     <col min="6" max="6" width="10.6640625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>433</v>
+        <v>421</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
@@ -5301,10 +5273,10 @@
         <v>39</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -5315,10 +5287,10 @@
         <v>42</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -5329,10 +5301,10 @@
         <v>44</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -5343,10 +5315,10 @@
         <v>46</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -5357,14 +5329,14 @@
         <v>48</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="F6" s="2"/>
     </row>
@@ -5373,17 +5345,17 @@
         <v>50</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -5391,17 +5363,17 @@
         <v>52</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -5409,17 +5381,17 @@
         <v>54</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>234</v>
+        <v>611</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
@@ -5427,10 +5399,10 @@
         <v>56</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -5438,710 +5410,710 @@
     </row>
     <row r="11" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>435</v>
+        <v>423</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>436</v>
+        <v>424</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2" t="s">
-        <v>439</v>
+        <v>427</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2" t="s">
-        <v>441</v>
+        <v>429</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
-        <v>442</v>
+        <v>430</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2" t="s">
-        <v>435</v>
+        <v>423</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2" t="s">
-        <v>443</v>
+        <v>431</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
-        <v>444</v>
+        <v>432</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2" t="s">
-        <v>435</v>
+        <v>423</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2" t="s">
-        <v>444</v>
+        <v>432</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
       <c r="F35" s="2" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2" t="s">
-        <v>259</v>
+        <v>610</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
       <c r="F37" s="2" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
       <c r="F38" s="2" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
       <c r="F39" s="2" t="s">
-        <v>444</v>
+        <v>432</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
       <c r="F40" s="2" t="s">
-        <v>445</v>
+        <v>433</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
       <c r="F41" s="2" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
       <c r="F42" s="2" t="s">
-        <v>444</v>
+        <v>432</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
       <c r="F43" s="2" t="s">
-        <v>444</v>
+        <v>432</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
       <c r="F44" s="2" t="s">
-        <v>444</v>
+        <v>432</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
       <c r="F45" s="2" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
       <c r="F46" s="2" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
       <c r="F47" s="2" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2" t="s">
-        <v>435</v>
+        <v>423</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="D49" s="2"/>
       <c r="E49" s="2" t="s">
-        <v>271</v>
+        <v>609</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>435</v>
+        <v>423</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="D50" s="2"/>
       <c r="E50" s="2"/>
       <c r="F50" s="2" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
       <c r="F51" s="2" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
       <c r="F52" s="2" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
       <c r="F53" s="2" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
       <c r="F54" s="2" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
     </row>
   </sheetData>
@@ -6180,7 +6152,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="58.109375" bestFit="1" customWidth="1"/>
@@ -6200,7 +6172,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -6208,7 +6180,7 @@
         <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -6217,143 +6189,127 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>57</v>
+        <v>605</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>452</v>
+        <v>597</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>60</v>
+        <v>263</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>453</v>
+        <v>70</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>276</v>
+        <v>606</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>93</v>
+        <v>598</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>155</v>
+        <v>607</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>446</v>
+        <v>599</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>159</v>
+        <v>608</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>447</v>
+        <v>600</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>202</v>
+        <v>265</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>448</v>
+        <v>601</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>206</v>
+        <v>266</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>449</v>
+        <v>602</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>210</v>
+        <v>267</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>450</v>
+        <v>603</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>214</v>
+        <v>268</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>451</v>
+        <v>604</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>454</v>
-      </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>455</v>
-      </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>456</v>
-      </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>457</v>
-      </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6381,7 +6337,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -6410,10 +6366,10 @@
         <v>10</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>12</v>
@@ -6424,1037 +6380,1037 @@
     </row>
     <row r="2" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2" t="s">
-        <v>499</v>
+        <v>475</v>
       </c>
       <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>500</v>
+        <v>476</v>
       </c>
       <c r="F3" s="1"/>
     </row>
     <row r="4" spans="1:6" ht="216" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>288</v>
+        <v>276</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>289</v>
+        <v>277</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
-        <v>501</v>
+        <v>477</v>
       </c>
       <c r="F4" s="1"/>
     </row>
     <row r="5" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>291</v>
+        <v>279</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>502</v>
+        <v>478</v>
       </c>
       <c r="F5" s="1"/>
     </row>
     <row r="6" spans="1:6" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>503</v>
+        <v>479</v>
       </c>
       <c r="F6" s="1"/>
     </row>
     <row r="7" spans="1:6" ht="144" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>504</v>
+        <v>480</v>
       </c>
       <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>505</v>
+        <v>481</v>
       </c>
       <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>505</v>
+        <v>481</v>
       </c>
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:6" ht="144" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>300</v>
+        <v>288</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>506</v>
+        <v>482</v>
       </c>
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" ht="144" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>506</v>
+        <v>482</v>
       </c>
       <c r="F11" s="1"/>
     </row>
     <row r="12" spans="1:6" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
-        <v>507</v>
+        <v>483</v>
       </c>
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2" t="s">
-        <v>508</v>
+        <v>484</v>
       </c>
       <c r="F13" s="1"/>
     </row>
     <row r="14" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
-        <v>509</v>
+        <v>485</v>
       </c>
       <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>510</v>
+        <v>486</v>
       </c>
       <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>511</v>
+        <v>487</v>
       </c>
       <c r="F16" s="1"/>
     </row>
     <row r="17" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
-        <v>512</v>
+        <v>488</v>
       </c>
       <c r="F17" s="1"/>
     </row>
     <row r="18" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
-        <v>513</v>
+        <v>489</v>
       </c>
       <c r="F18" s="1"/>
     </row>
     <row r="19" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
-        <v>514</v>
+        <v>490</v>
       </c>
       <c r="F19" s="1"/>
     </row>
     <row r="20" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2" t="s">
-        <v>515</v>
+        <v>491</v>
       </c>
       <c r="F20" s="1"/>
     </row>
     <row r="21" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2" t="s">
-        <v>516</v>
+        <v>492</v>
       </c>
       <c r="F21" s="1"/>
     </row>
     <row r="22" spans="1:6" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2" t="s">
-        <v>517</v>
+        <v>493</v>
       </c>
       <c r="F22" s="1"/>
     </row>
     <row r="23" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2" t="s">
-        <v>518</v>
+        <v>494</v>
       </c>
       <c r="F23" s="1"/>
     </row>
     <row r="24" spans="1:6" ht="360" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2" t="s">
-        <v>519</v>
+        <v>495</v>
       </c>
       <c r="F24" s="1"/>
     </row>
     <row r="25" spans="1:6" ht="216" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2" t="s">
-        <v>520</v>
+        <v>496</v>
       </c>
       <c r="F25" s="1"/>
     </row>
     <row r="26" spans="1:6" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2" t="s">
-        <v>521</v>
+        <v>497</v>
       </c>
       <c r="F26" s="1"/>
     </row>
     <row r="27" spans="1:6" ht="144" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2" t="s">
-        <v>522</v>
+        <v>498</v>
       </c>
       <c r="F27" s="1"/>
     </row>
     <row r="28" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2" t="s">
-        <v>523</v>
+        <v>499</v>
       </c>
       <c r="F28" s="1"/>
     </row>
     <row r="29" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2" t="s">
-        <v>524</v>
+        <v>500</v>
       </c>
       <c r="F29" s="1"/>
     </row>
     <row r="30" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2" t="s">
-        <v>525</v>
+        <v>501</v>
       </c>
       <c r="F30" s="1"/>
     </row>
     <row r="31" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2" t="s">
-        <v>526</v>
+        <v>502</v>
       </c>
       <c r="F31" s="1"/>
     </row>
     <row r="32" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2" t="s">
-        <v>527</v>
+        <v>503</v>
       </c>
       <c r="F32" s="1"/>
     </row>
     <row r="33" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2" t="s">
-        <v>528</v>
+        <v>504</v>
       </c>
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="1:6" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2" t="s">
-        <v>529</v>
+        <v>505</v>
       </c>
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2" t="s">
-        <v>530</v>
+        <v>506</v>
       </c>
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2" t="s">
-        <v>531</v>
+        <v>507</v>
       </c>
       <c r="F36" s="1"/>
     </row>
     <row r="37" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2" t="s">
-        <v>530</v>
+        <v>506</v>
       </c>
       <c r="F37" s="1"/>
     </row>
     <row r="38" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2" t="s">
-        <v>531</v>
+        <v>507</v>
       </c>
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2" t="s">
-        <v>532</v>
+        <v>508</v>
       </c>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>533</v>
+        <v>509</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2" t="s">
-        <v>532</v>
+        <v>508</v>
       </c>
       <c r="F41" s="1"/>
     </row>
     <row r="42" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2" t="s">
-        <v>533</v>
+        <v>509</v>
       </c>
       <c r="F42" s="1"/>
     </row>
     <row r="43" spans="1:6" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2" t="s">
-        <v>534</v>
+        <v>510</v>
       </c>
       <c r="F43" s="1"/>
     </row>
     <row r="44" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2" t="s">
-        <v>535</v>
+        <v>511</v>
       </c>
       <c r="F44" s="1"/>
     </row>
     <row r="45" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2" t="s">
-        <v>536</v>
+        <v>512</v>
       </c>
       <c r="F45" s="1"/>
     </row>
     <row r="46" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2" t="s">
-        <v>537</v>
+        <v>513</v>
       </c>
       <c r="F46" s="1"/>
     </row>
     <row r="47" spans="1:6" ht="216" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2" t="s">
-        <v>538</v>
+        <v>514</v>
       </c>
       <c r="F47" s="1"/>
     </row>
     <row r="48" spans="1:6" ht="144" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2" t="s">
-        <v>539</v>
+        <v>515</v>
       </c>
       <c r="F48" s="1"/>
     </row>
     <row r="49" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2" t="s">
-        <v>540</v>
+        <v>516</v>
       </c>
       <c r="F49" s="1"/>
     </row>
     <row r="50" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2" t="s">
-        <v>541</v>
+        <v>517</v>
       </c>
       <c r="F50" s="1"/>
     </row>
     <row r="51" spans="1:6" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>382</v>
+        <v>370</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>383</v>
+        <v>371</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2" t="s">
-        <v>542</v>
+        <v>518</v>
       </c>
       <c r="F51" s="1"/>
     </row>
     <row r="52" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>384</v>
+        <v>372</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>385</v>
+        <v>373</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2" t="s">
-        <v>543</v>
+        <v>519</v>
       </c>
       <c r="F52" s="1"/>
     </row>
     <row r="53" spans="1:6" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>386</v>
+        <v>374</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>387</v>
+        <v>375</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2" t="s">
-        <v>544</v>
+        <v>520</v>
       </c>
       <c r="F53" s="1"/>
     </row>
     <row r="54" spans="1:6" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>388</v>
+        <v>376</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>389</v>
+        <v>377</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2" t="s">
-        <v>545</v>
+        <v>521</v>
       </c>
       <c r="F54" s="1"/>
     </row>
     <row r="55" spans="1:6" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2" t="s">
-        <v>546</v>
+        <v>522</v>
       </c>
       <c r="F55" s="1"/>
     </row>
     <row r="56" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2" t="s">
-        <v>547</v>
+        <v>523</v>
       </c>
       <c r="F56" s="1"/>
     </row>
     <row r="57" spans="1:6" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>394</v>
+        <v>382</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2" t="s">
-        <v>548</v>
+        <v>524</v>
       </c>
       <c r="F57" s="1"/>
     </row>
     <row r="58" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>397</v>
+        <v>385</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
       <c r="E58" s="2" t="s">
-        <v>549</v>
+        <v>525</v>
       </c>
       <c r="F58" s="1"/>
     </row>
     <row r="59" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>398</v>
+        <v>386</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>399</v>
+        <v>387</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
       <c r="E59" s="2" t="s">
-        <v>550</v>
+        <v>526</v>
       </c>
       <c r="F59" s="1"/>
     </row>
     <row r="60" spans="1:6" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>400</v>
+        <v>388</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>401</v>
+        <v>389</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="2" t="s">
-        <v>551</v>
+        <v>527</v>
       </c>
       <c r="F60" s="1"/>
     </row>
     <row r="61" spans="1:6" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>402</v>
+        <v>390</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
       <c r="E61" s="2" t="s">
-        <v>552</v>
+        <v>528</v>
       </c>
       <c r="F61" s="1"/>
     </row>
     <row r="62" spans="1:6" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>404</v>
+        <v>392</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
       <c r="E62" s="2" t="s">
-        <v>553</v>
+        <v>529</v>
       </c>
       <c r="F62" s="1"/>
     </row>
     <row r="63" spans="1:6" ht="216" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>406</v>
+        <v>394</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>407</v>
+        <v>395</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
       <c r="E63" s="2" t="s">
-        <v>554</v>
+        <v>530</v>
       </c>
       <c r="F63" s="1"/>
     </row>
     <row r="64" spans="1:6" ht="144" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>408</v>
+        <v>396</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>409</v>
+        <v>397</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
       <c r="E64" s="2" t="s">
-        <v>555</v>
+        <v>531</v>
       </c>
       <c r="F64" s="1"/>
     </row>
     <row r="65" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>410</v>
+        <v>398</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>411</v>
+        <v>399</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
       <c r="E65" s="2" t="s">
-        <v>556</v>
+        <v>532</v>
       </c>
       <c r="F65" s="1"/>
     </row>
     <row r="66" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>412</v>
+        <v>400</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>413</v>
+        <v>401</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
       <c r="E66" s="2" t="s">
-        <v>557</v>
+        <v>533</v>
       </c>
       <c r="F66" s="1"/>
     </row>
     <row r="67" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
-        <v>414</v>
+        <v>402</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>415</v>
+        <v>403</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
       <c r="E67" s="2" t="s">
-        <v>558</v>
+        <v>534</v>
       </c>
       <c r="F67" s="1"/>
     </row>
     <row r="68" spans="1:6" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
-        <v>416</v>
+        <v>404</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>417</v>
+        <v>405</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
       <c r="E68" s="2" t="s">
-        <v>559</v>
+        <v>535</v>
       </c>
       <c r="F68" s="1"/>
     </row>
     <row r="69" spans="1:6" ht="144" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>418</v>
+        <v>406</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>419</v>
+        <v>407</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" s="2"/>
       <c r="E69" s="2" t="s">
-        <v>560</v>
+        <v>536</v>
       </c>
       <c r="F69" s="1"/>
     </row>
     <row r="70" spans="1:6" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>421</v>
+        <v>409</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" s="2"/>
       <c r="E70" s="2" t="s">
-        <v>561</v>
+        <v>537</v>
       </c>
       <c r="F70" s="1"/>
     </row>
     <row r="71" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>423</v>
+        <v>411</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" s="2"/>
       <c r="E71" s="2" t="s">
-        <v>562</v>
+        <v>538</v>
       </c>
       <c r="F71" s="1"/>
     </row>
     <row r="72" spans="1:6" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>424</v>
+        <v>412</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>421</v>
+        <v>409</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
       <c r="E72" s="2" t="s">
-        <v>561</v>
+        <v>537</v>
       </c>
       <c r="F72" s="1"/>
     </row>
     <row r="73" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>425</v>
+        <v>413</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>423</v>
+        <v>411</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
       <c r="E73" s="2" t="s">
-        <v>562</v>
+        <v>538</v>
       </c>
       <c r="F73" s="1"/>
     </row>
     <row r="74" spans="1:6" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
-        <v>426</v>
+        <v>414</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>427</v>
+        <v>415</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" s="2"/>
       <c r="E74" s="2" t="s">
-        <v>563</v>
+        <v>539</v>
       </c>
       <c r="F74" s="1"/>
     </row>
     <row r="75" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
-        <v>428</v>
+        <v>416</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>429</v>
+        <v>417</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
       <c r="E75" s="2" t="s">
-        <v>564</v>
+        <v>540</v>
       </c>
       <c r="F75" s="1"/>
     </row>

</xml_diff>